<commit_message>
docs: CW22 session logs — 7 Excel + 7 doc sync + cross-verification
- Work Log (2603292100): 21-row timeline of signup flow fixes
- Cowork Log (CW22-B): 16-row session dialogue
- D9/D10/D12/D14/D15 Excel updates
- CLAUDE.md, CHANGELOG.md, NEXT_SESSION_START.md, DIVISION_STATUS.md,
  COWORK_SESSION_HISTORY.md all synced to 22:00 KST

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/POTAL_D10_Revenue_Billing.xlsx
+++ b/POTAL_D10_Revenue_Billing.xlsx
@@ -7,12 +7,13 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="CW21_20260328" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="구독현황" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="MRR추이" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Overage정산" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Paddle이벤트" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="D10 Dashboard" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="CW22B_NoChange" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="CW21_20260328" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="구독현황" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="MRR추이" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Overage정산" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Paddle이벤트" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="D10 Dashboard" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -512,6 +513,84 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" style="11" min="1" max="1"/>
+    <col width="70" customWidth="1" style="11" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="23" t="inlineStr">
+        <is>
+          <t>항목</t>
+        </is>
+      </c>
+      <c r="B1" s="23" t="inlineStr">
+        <is>
+          <t>내용</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>날짜</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-03-29 21:00 KST</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>변경사항</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>없음 — Forever Free 구조 유지</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>확인</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>가입 플로우에서 plan_id: 'free', subscription_status: 'active' 자동 설정</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>MRR</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>$0 (의도적 — Exit 전략)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -544,44 +623,44 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>2026-03-28 23:30 KST</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="10" t="inlineStr">
         <is>
           <t>v3 파이프라인 완성</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="10" t="inlineStr">
         <is>
           <t>21/21 Section 100%, AI 0회 호출</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="10" t="inlineStr">
         <is>
           <t>API 당 비용 $0 유지 → 마진 100%</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>2026-03-28 23:30 KST</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="10" t="inlineStr">
         <is>
           <t>정확도 개선</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="10" t="inlineStr">
         <is>
           <t>22/22 regression PASS</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="10" t="inlineStr">
         <is>
           <t>과금 가능한 품질 수준 달성</t>
         </is>
@@ -592,7 +671,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -692,7 +771,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1057,7 +1136,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1145,7 +1224,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1233,7 +1312,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>